<commit_message>
Actualización automática de base de datos
</commit_message>
<xml_diff>
--- a/LMI Base.xlsx
+++ b/LMI Base.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Semith Kiliçsoy</t>
+          <t>Semih Kılıçsoy</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Samu Aghehowa</t>
+          <t>Samu Omorodion</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>K. Kvaratskhelia</t>
+          <t>Khvicha Kvaratskhelia</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>C. Summerville</t>
+          <t>Crysencio Summerville</t>
         </is>
       </c>
       <c r="C48" s="3" t="n">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Kenan Yildiz</t>
+          <t>Kenan Yıldız</t>
         </is>
       </c>
       <c r="C55" s="3" t="n">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Baris Alper Yılmaz</t>
+          <t>Barış Alper Yılmaz</t>
         </is>
       </c>
       <c r="C92" s="3" t="n">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Ferdi Kadioğlu</t>
+          <t>Ferdi Kadıoğlu</t>
         </is>
       </c>
       <c r="C146" s="3" t="n"/>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Jakud Kiwior</t>
+          <t>Jakub Kiwior</t>
         </is>
       </c>
       <c r="C154" s="3" t="n"/>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>T. Alexander-Arnold</t>
+          <t>Trent Alexander-Arnold</t>
         </is>
       </c>
       <c r="C158" s="3" t="n"/>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>Alex Zendejas</t>
+          <t>Alejandro Zendejas</t>
         </is>
       </c>
       <c r="C161" s="3" t="n"/>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Bruno Fernandez</t>
+          <t>Bruno Fernandes</t>
         </is>
       </c>
       <c r="C181" s="3" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Semith Kiliçsoy</t>
+          <t>Semih Kılıçsoy</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Kenan Yildiz</t>
+          <t>Kenan Yıldız</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>C. Summerville</t>
+          <t>Crysencio Summerville</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>K. Kvaratskhelia</t>
+          <t>Khvicha Kvaratskhelia</t>
         </is>
       </c>
       <c r="C58" s="3" t="n">
@@ -8621,7 +8621,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Alex Zendejas</t>
+          <t>Alejandro Zendejas</t>
         </is>
       </c>
       <c r="C81" s="3" t="n"/>
@@ -10355,7 +10355,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Arda Güler (P)</t>
+          <t>Arda Güler</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">

</xml_diff>